<commit_message>
cambios finales eso espero
</commit_message>
<xml_diff>
--- a/Llamen a Dios/Resources/Plantilla Cierre de Caja.xlsx
+++ b/Llamen a Dios/Resources/Plantilla Cierre de Caja.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sonku\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE1CA807-CCE0-41E0-8ECB-1E80C68256D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F145A137-6F8C-4875-A72D-076B493D5589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{3E226D24-DF79-48D7-B4DA-EDFDB0A00578}"/>
   </bookViews>
@@ -69,19 +69,19 @@
     <t>PAN DE PARÍS C.A</t>
   </si>
   <si>
-    <t>Generado: 03/07/2026 05:26 PM</t>
-  </si>
-  <si>
     <t>Por:</t>
   </si>
   <si>
-    <t>Direccion:</t>
-  </si>
-  <si>
     <t>Movimientos de Productos</t>
   </si>
   <si>
     <t xml:space="preserve">Generado: </t>
+  </si>
+  <si>
+    <t>Direccion: Av Jóvito Villalba, 6316, Nueva Esparta</t>
+  </si>
+  <si>
+    <t>Direccion:  Av Jóvito Villalba, 6316, Nueva Esparta</t>
   </si>
 </sst>
 </file>
@@ -170,7 +170,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -181,28 +181,25 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -296,8 +293,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>179711</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1292231</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>15240</xdr:rowOff>
     </xdr:to>
@@ -658,125 +655,143 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A7FCEFA-00B3-498A-9D84-5C02412A1246}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.109375" customWidth="1"/>
-    <col min="2" max="2" width="30.109375" customWidth="1"/>
-    <col min="3" max="3" width="27.5546875" customWidth="1"/>
+    <col min="2" max="2" width="19.109375" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" customWidth="1"/>
     <col min="4" max="4" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D1" s="2"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="D2" s="2"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B3" s="2" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D3" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="2"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B4" s="10" t="s">
+      <c r="E3" s="9"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D4" s="8" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B5" s="12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B6" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B7" t="s">
+      <c r="E4" s="8"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C5" s="11" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="9" t="s">
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C6" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C7" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="9"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
+      <c r="B10" s="10"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="6"/>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="5"/>
       <c r="B12" s="3"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="7"/>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B13" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="6">
+    <mergeCell ref="C7:E7"/>
     <mergeCell ref="A10:B10"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="C5:E5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9431875D-9F75-4D8B-B893-DE45FBD004C7}">
-  <dimension ref="A2:D12"/>
+  <dimension ref="A2:E12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.5546875" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" customWidth="1"/>
     <col min="2" max="2" width="22.21875" customWidth="1"/>
     <col min="3" max="3" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.44140625" customWidth="1"/>
+    <col min="4" max="4" width="16.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C2" s="8" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D2" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="8"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C3" s="11" t="s">
+      <c r="E2" s="9"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="11"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C4" s="8" t="s">
+      <c r="E3" s="8"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C4" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C5" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="8"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C5" t="s">
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C6" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+    </row>
+    <row r="9" spans="1:5" ht="18" x14ac:dyDescent="0.35">
+      <c r="A9" s="7" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="18" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>3</v>
       </c>
@@ -790,20 +805,23 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
     <mergeCell ref="A9:D9"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="C4:E4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>